<commit_message>
Save local workspace changes and push updates to origin
</commit_message>
<xml_diff>
--- a/menu_prompt_documentation.xlsx
+++ b/menu_prompt_documentation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\spandana\OneDrive\Desktop\New Menu Recomendation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/12ee2bda9bec77cf/Desktop/New Menu Recomendation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA7712E-1C14-496D-BC95-35B8C77B4F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{5EA7712E-1C14-496D-BC95-35B8C77B4F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6A4AB0A-44C4-41EF-8244-3857436792F7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -150,6 +150,12 @@
   </si>
   <si>
     <t>AI customer intelligence data generation</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Insights</t>
   </si>
   <si>
     <t>Generate NEW MENU RECOMMENDATIONS for all restaurants using only the available dataset.
@@ -266,58 +272,102 @@
 - Avoid repetitive dishes across restaurants
 - Recommendations must feel unique to each restaurant, location, demographic cluster, and cuisine ecosystem
 Generate realistic and context-aware values for:
-- demographic_segmentation
-- restaurant_type
-- market_segment
-- health_type
-- cuisine_type
-- dominant_ethnicity
-- target_customer_segment
-- target_audience
-- why_this_will_work
-- recommended_menu
-Target customer segment should intelligently combine:
-- age behavior
-- family behavior
-- premium behavior
-- wellness behavior
-- spending behavior
-- dining behavior
-Each restaurant should receive maximum 6–7 menu recommendations.
-Recommended menu may include:
-- appetizers
-- snacks
-- bowls
-- beverages
-- healthy meals
-- combo meals
-- premium dishes
-- regional fusion dishes
-- signature dishes
-Final Output:
-Return the fully updated CSV/Excel dataset with these generated columns populated automatically for every restaurant:
-- restaurant_name (direcly fetch from the file attached)
-- restaurant_object_key (direcly fetch from the file attached)
-- zip_or_postal_code (direcly fetch from the file attached)
-- city (direcly fetch from the file attached)
-- state (direcly fetch from the file attached)
-- county (direcly fetch from the file attached)
-- demographic_segmentation (direcly fetch from the file attached)
-- restaurant category(direcly fetch from the file attached)
-- market_segment (direcly fetch from the file attached)
-- health_type (direcly fetch from the file attached)
-- taste_features(direcly fetch from the file attached)
-- dominant_ethnicity (direcly fetch from the file attached)
-- target_customer_segment (direcly fetch from the file attached)
-- target_audience 
-- why_this_will_work
-- recommended_menu</t>
-  </si>
-  <si>
-    <t>Result</t>
-  </si>
-  <si>
-    <t>Insights</t>
+NEW MENU RECOMMENDATION   ACROSS MEMPHIS  
+he recommendation engine should generate thousands of different menu combinations across Memphis, not one Memphis menu repeated for every restaurant. The menu must be driven by the actual intelligence columns in the dataset, with city/ZIP intelligence influencing demand and restaurant category acting as a validation layer rather than a fixed template.
+PRIORITY ORDER
+1. City
+2. Region
+3. State
+4. Local demographics
+5. Customer intelligence
+6. AI-generated customer reviews and feedback
+7. Food preference trends
+8. Health and wellness trends
+9. Restaurant category
+MENU RECOMMENDATION LOGIC
+For each restaurant, first analyze the available columns from merged_customer_intelligence.xlsx.
+The engine must understand:
+* City-level food behavior
+* Regional cuisine preferences
+* Population characteristics
+* Income and spending behavior
+* Family composition
+* Age distribution
+* Health-conscious consumer behavior
+* Premium dining demand
+* Convenience demand
+* Local food trends
+* Customer sentiment
+* AI-generated review intelligence
+* Cuisine affinity
+* Flavor preferences
+* Portion-size expectations
+* Price sensitivity
+* Ordering behavior
+The engine must use the demographic and customer intelligence data to determine what customers in that ZIP code, city, and region are most likely to purchase.
+Customer review intelligence should strongly influence menu creation.
+Generated reviews should reveal:
+* Foods customers enjoy most
+* Common complaints
+* Desired menu additions
+* Health-related requests
+* Premium food demand
+* Family meal demand
+* Convenience demand
+* Flavor preferences
+* Protein preferences
+* Beverage preferences
+Only after understanding the above intelligence should the engine apply restaurant-category rules.
+CATEGORY-BASED RECOMMENDATION INTELLIGENCE
+The recommendation engine must generate dishes that naturally fit the restaurant business model, customer expectations, cuisine behavior, pricing style, serving style, and dining behavior.
+Restaurant Category Intelligence
+Use the restaurant category provided in the dataset as a contextual guide rather than a rigid menu template.
+The recommendation engine should:
+* Prioritize ZCTA, city, regional, and local market intelligence to understand customer preferences, purchasing behavior, and food demand patterns.
+* Ensure recommended menu items align with the restaurant category.
+* Adapt menu recommendations based on location intelligence, demographics, customer intelligence, review intelligence, and trend intelligence.
+* Allow regional and customer-driven preferences to influence menu composition.
+* Balance category relevance with local demand and customer behavior.
+* Generate menu items that feel authentic to both the restaurant concept and the surrounding market.
+Regional, demographic, and customer-review intelligence should be the primary drivers of menu recommendations. The engine must prioritize city, region, state, local demographics, customer behavior insights, and AI-generated customer reviews to understand what customers in that area are most likely to order. Restaurant category should be used only to ensure the recommendations fit the restaurant’s business model and menu style, without overriding stronger signals from regional preferences, demographic trends, or customer feedback.
+CATEGORY DOMINANCE RULES
+Restaurant category behavior must dominate:
+* Dish naming
+* Ingredient selection
+* Flavor profile
+* Cooking style
+* Pricing perception
+* Serving format
+* Target audience
+* Menu structure
+* Trend adaptation
+* Health adaptation
+* Portion sizing
+* Customization behavior
+STRICT RULE
+Do not generate dishes that conflict with the restaurant category.this is ZCTA/ regoinal based withe cosidaration of1. City
+2. Region
+3. State
+4. Local demographics
+5. Customer intelligence
+6. AI-generated customer reviews and feedback
+7. Food preference trends
+8. Health and wellness trends
+9. Restaurant category
+FINAL DECISION RULE
+Menu recommendations must be generated by combining:
+Location Intelligence (City + Region + State)
++
+Demographic Intelligence
++
+Customer Intelligence
++
+AI-Generated Review Intelligence
++
+Food Trend Intelligence
++
+Restaurant Category Intelligence
+The final menu should feel like a menu that customers in that specific location would naturally order . and give .xlsx format</t>
   </si>
 </sst>
 </file>
@@ -744,10 +794,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>6</v>
@@ -764,7 +814,7 @@
         <v>25</v>
       </c>
       <c r="C2" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>9</v>
@@ -787,10 +837,10 @@
         <v>24</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C3" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>9</v>

</xml_diff>